<commit_message>
Update: WMiranda_2026TimeTracking.xlsx [2026-04-14 13:34 UTC]
</commit_message>
<xml_diff>
--- a/WMiranda_2026TimeTracking.xlsx
+++ b/WMiranda_2026TimeTracking.xlsx
@@ -7340,7 +7340,9 @@
         <v>1.5</v>
       </c>
       <c r="BW9" s="32" t="n"/>
-      <c r="BX9" s="32" t="n"/>
+      <c r="BX9" s="32" t="n">
+        <v>0.5</v>
+      </c>
       <c r="BY9" s="32" t="n"/>
       <c r="BZ9" s="32" t="n"/>
       <c r="CA9" s="32" t="n"/>

</xml_diff>

<commit_message>
Update: WMiranda_2026TimeTracking.xlsx [2026-04-14 16:59 UTC]
</commit_message>
<xml_diff>
--- a/WMiranda_2026TimeTracking.xlsx
+++ b/WMiranda_2026TimeTracking.xlsx
@@ -14108,7 +14108,9 @@
       <c r="BW33" s="32" t="n">
         <v>3</v>
       </c>
-      <c r="BX33" s="32" t="n"/>
+      <c r="BX33" s="32" t="n">
+        <v>4</v>
+      </c>
       <c r="BY33" s="32" t="n"/>
       <c r="BZ33" s="32" t="n"/>
       <c r="CA33" s="32" t="n"/>

</xml_diff>

<commit_message>
Update: WMiranda_2026TimeTracking.xlsx [2026-04-15 20:22 UTC]
</commit_message>
<xml_diff>
--- a/WMiranda_2026TimeTracking.xlsx
+++ b/WMiranda_2026TimeTracking.xlsx
@@ -7343,7 +7343,9 @@
       <c r="BX9" s="32" t="n">
         <v>0.5</v>
       </c>
-      <c r="BY9" s="32" t="n"/>
+      <c r="BY9" s="32" t="n">
+        <v>1</v>
+      </c>
       <c r="BZ9" s="32" t="n"/>
       <c r="CA9" s="32" t="n"/>
       <c r="CB9" s="32" t="n"/>
@@ -7927,7 +7929,9 @@
         <v>1</v>
       </c>
       <c r="BX11" s="17" t="n"/>
-      <c r="BY11" s="17" t="n"/>
+      <c r="BY11" s="17" t="n">
+        <v>0.5</v>
+      </c>
       <c r="BZ11" s="17" t="n"/>
       <c r="CA11" s="17" t="n"/>
       <c r="CB11" s="17" t="n"/>
@@ -9643,7 +9647,9 @@
       <c r="BV17" s="32" t="n"/>
       <c r="BW17" s="32" t="n"/>
       <c r="BX17" s="32" t="n"/>
-      <c r="BY17" s="32" t="n"/>
+      <c r="BY17" s="32" t="n">
+        <v>1.5</v>
+      </c>
       <c r="BZ17" s="32" t="n"/>
       <c r="CA17" s="32" t="n"/>
       <c r="CB17" s="32" t="n"/>
@@ -14111,7 +14117,9 @@
       <c r="BX33" s="32" t="n">
         <v>4</v>
       </c>
-      <c r="BY33" s="32" t="n"/>
+      <c r="BY33" s="32" t="n">
+        <v>2</v>
+      </c>
       <c r="BZ33" s="32" t="n"/>
       <c r="CA33" s="32" t="n"/>
       <c r="CB33" s="32" t="n"/>
@@ -23795,7 +23803,9 @@
         <v>1.5</v>
       </c>
       <c r="BX68" s="32" t="n"/>
-      <c r="BY68" s="32" t="n"/>
+      <c r="BY68" s="32" t="n">
+        <v>3.5</v>
+      </c>
       <c r="BZ68" s="32" t="n"/>
       <c r="CA68" s="32" t="n"/>
       <c r="CB68" s="32" t="n"/>

</xml_diff>

<commit_message>
Sync from OneDrive: WMiranda_2026TimeTracking.xlsx [2026-04-15 22:00 UTC]
</commit_message>
<xml_diff>
--- a/WMiranda_2026TimeTracking.xlsx
+++ b/WMiranda_2026TimeTracking.xlsx
@@ -31019,4 +31019,277 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008A7894324D7C3949B4D325554D1FC6DA" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="43dd22c4a0a55be49439aa2cba9a6031">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="be2d32d5-45e4-45f8-8cca-e731efdae529" xmlns:ns3="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="67300191881baa0ec8105967d66c0489" ns2:_="" ns3:_="">
+    <xsd:import namespace="be2d32d5-45e4-45f8-8cca-e731efdae529"/>
+    <xsd:import namespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="be2d32d5-45e4-45f8-8cca-e731efdae529" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="10" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="11" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="7ff297e6-98dc-4a77-8782-4199b303df17" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="17" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="20" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="21" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="22" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="23" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{433bb87c-b111-4230-a796-99831eb60517}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="be2d32d5-45e4-45f8-8cca-e731efdae529">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{48EF5A99-86E2-4ECD-8F5E-0EC6695B5C21}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1C67DED5-99DE-4140-A1FB-C2F1D56A3D5E}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{16374960-44BF-44AC-A60C-72CA894C3392}"/>
 </file>
</xml_diff>

<commit_message>
Update: WMiranda_2026TimeTracking.xlsx [2026-04-16 19:24 UTC]
</commit_message>
<xml_diff>
--- a/WMiranda_2026TimeTracking.xlsx
+++ b/WMiranda_2026TimeTracking.xlsx
@@ -7346,7 +7346,9 @@
       <c r="BY9" s="32" t="n">
         <v>1</v>
       </c>
-      <c r="BZ9" s="32" t="n"/>
+      <c r="BZ9" s="32" t="n">
+        <v>0.75</v>
+      </c>
       <c r="CA9" s="32" t="n"/>
       <c r="CB9" s="32" t="n"/>
       <c r="CC9" s="32" t="n"/>
@@ -9650,7 +9652,9 @@
       <c r="BY17" s="32" t="n">
         <v>1.5</v>
       </c>
-      <c r="BZ17" s="32" t="n"/>
+      <c r="BZ17" s="32" t="n">
+        <v>1.75</v>
+      </c>
       <c r="CA17" s="32" t="n"/>
       <c r="CB17" s="32" t="n"/>
       <c r="CC17" s="32" t="n"/>
@@ -10214,7 +10218,9 @@
       <c r="BW19" s="17" t="n"/>
       <c r="BX19" s="17" t="n"/>
       <c r="BY19" s="17" t="n"/>
-      <c r="BZ19" s="17" t="n"/>
+      <c r="BZ19" s="17" t="n">
+        <v>1</v>
+      </c>
       <c r="CA19" s="17" t="n"/>
       <c r="CB19" s="17" t="n"/>
       <c r="CC19" s="17" t="n"/>
@@ -14120,7 +14126,9 @@
       <c r="BY33" s="32" t="n">
         <v>2</v>
       </c>
-      <c r="BZ33" s="32" t="n"/>
+      <c r="BZ33" s="32" t="n">
+        <v>2</v>
+      </c>
       <c r="CA33" s="32" t="n"/>
       <c r="CB33" s="32" t="n"/>
       <c r="CC33" s="32" t="n"/>
@@ -21791,7 +21799,9 @@
       <c r="BW61" s="17" t="n"/>
       <c r="BX61" s="17" t="n"/>
       <c r="BY61" s="17" t="n"/>
-      <c r="BZ61" s="17" t="n"/>
+      <c r="BZ61" s="17" t="n">
+        <v>1.75</v>
+      </c>
       <c r="CA61" s="17" t="n"/>
       <c r="CB61" s="17" t="n"/>
       <c r="CC61" s="17" t="n"/>
@@ -23806,7 +23816,9 @@
       <c r="BY68" s="32" t="n">
         <v>3.5</v>
       </c>
-      <c r="BZ68" s="32" t="n"/>
+      <c r="BZ68" s="32" t="n">
+        <v>1.25</v>
+      </c>
       <c r="CA68" s="32" t="n"/>
       <c r="CB68" s="32" t="n"/>
       <c r="CC68" s="32" t="n"/>
@@ -26322,7 +26334,9 @@
       <c r="BW77" s="17" t="n"/>
       <c r="BX77" s="17" t="n"/>
       <c r="BY77" s="17" t="n"/>
-      <c r="BZ77" s="17" t="n"/>
+      <c r="BZ77" s="17" t="n">
+        <v>1</v>
+      </c>
       <c r="CA77" s="17" t="n"/>
       <c r="CB77" s="17" t="n"/>
       <c r="CC77" s="17" t="n"/>
@@ -31019,277 +31033,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008A7894324D7C3949B4D325554D1FC6DA" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="43dd22c4a0a55be49439aa2cba9a6031">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="be2d32d5-45e4-45f8-8cca-e731efdae529" xmlns:ns3="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="67300191881baa0ec8105967d66c0489" ns2:_="" ns3:_="">
-    <xsd:import namespace="be2d32d5-45e4-45f8-8cca-e731efdae529"/>
-    <xsd:import namespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="be2d32d5-45e4-45f8-8cca-e731efdae529" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="10" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="11" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="7ff297e6-98dc-4a77-8782-4199b303df17" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="17" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="20" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="21" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="22" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="23" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{433bb87c-b111-4230-a796-99831eb60517}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="be2d32d5-45e4-45f8-8cca-e731efdae529">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{48EF5A99-86E2-4ECD-8F5E-0EC6695B5C21}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1C67DED5-99DE-4140-A1FB-C2F1D56A3D5E}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{16374960-44BF-44AC-A60C-72CA894C3392}"/>
 </file>
</xml_diff>

<commit_message>
Sync from OneDrive: WMiranda_2026TimeTracking.xlsx [2026-04-16 21:00 UTC]
</commit_message>
<xml_diff>
--- a/WMiranda_2026TimeTracking.xlsx
+++ b/WMiranda_2026TimeTracking.xlsx
@@ -31033,4 +31033,277 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008A7894324D7C3949B4D325554D1FC6DA" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="43dd22c4a0a55be49439aa2cba9a6031">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="be2d32d5-45e4-45f8-8cca-e731efdae529" xmlns:ns3="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="67300191881baa0ec8105967d66c0489" ns2:_="" ns3:_="">
+    <xsd:import namespace="be2d32d5-45e4-45f8-8cca-e731efdae529"/>
+    <xsd:import namespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="be2d32d5-45e4-45f8-8cca-e731efdae529" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="10" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="11" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="7ff297e6-98dc-4a77-8782-4199b303df17" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="17" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="20" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="21" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="22" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="23" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{433bb87c-b111-4230-a796-99831eb60517}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="be2d32d5-45e4-45f8-8cca-e731efdae529">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{552BB8D9-DC48-4340-BCF7-4C1B635CEC7F}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00E3C019-928C-4C37-A671-BB9F14B50437}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1440C824-587B-4F41-8DE4-A8B2A9A677C8}"/>
 </file>
</xml_diff>

<commit_message>
Update: WMiranda_2026TimeTracking.xlsx [2026-04-20 21:07 UTC]
</commit_message>
<xml_diff>
--- a/WMiranda_2026TimeTracking.xlsx
+++ b/WMiranda_2026TimeTracking.xlsx
@@ -7350,7 +7350,9 @@
         <v>0.75</v>
       </c>
       <c r="CA9" s="32" t="n"/>
-      <c r="CB9" s="32" t="n"/>
+      <c r="CB9" s="32" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CC9" s="32" t="n"/>
       <c r="CD9" s="32" t="n"/>
       <c r="CE9" s="32" t="n"/>
@@ -7936,7 +7938,9 @@
       </c>
       <c r="BZ11" s="17" t="n"/>
       <c r="CA11" s="17" t="n"/>
-      <c r="CB11" s="17" t="n"/>
+      <c r="CB11" s="17" t="n">
+        <v>1.25</v>
+      </c>
       <c r="CC11" s="17" t="n"/>
       <c r="CD11" s="17" t="n"/>
       <c r="CE11" s="17" t="n"/>
@@ -8208,7 +8212,9 @@
       <c r="BY12" s="17" t="n"/>
       <c r="BZ12" s="17" t="n"/>
       <c r="CA12" s="17" t="n"/>
-      <c r="CB12" s="17" t="n"/>
+      <c r="CB12" s="17" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CC12" s="17" t="n"/>
       <c r="CD12" s="17" t="n"/>
       <c r="CE12" s="17" t="n"/>
@@ -9656,7 +9662,9 @@
         <v>1.75</v>
       </c>
       <c r="CA17" s="32" t="n"/>
-      <c r="CB17" s="32" t="n"/>
+      <c r="CB17" s="32" t="n">
+        <v>5</v>
+      </c>
       <c r="CC17" s="32" t="n"/>
       <c r="CD17" s="32" t="n"/>
       <c r="CE17" s="32" t="n"/>
@@ -14130,7 +14138,9 @@
         <v>2</v>
       </c>
       <c r="CA33" s="32" t="n"/>
-      <c r="CB33" s="32" t="n"/>
+      <c r="CB33" s="32" t="n">
+        <v>1</v>
+      </c>
       <c r="CC33" s="32" t="n"/>
       <c r="CD33" s="32" t="n"/>
       <c r="CE33" s="32" t="n"/>
@@ -18791,7 +18801,9 @@
       <c r="BY50" s="17" t="n"/>
       <c r="BZ50" s="17" t="n"/>
       <c r="CA50" s="17" t="n"/>
-      <c r="CB50" s="17" t="n"/>
+      <c r="CB50" s="17" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CC50" s="17" t="n"/>
       <c r="CD50" s="17" t="n"/>
       <c r="CE50" s="17" t="n"/>
@@ -23820,7 +23832,9 @@
         <v>1.25</v>
       </c>
       <c r="CA68" s="32" t="n"/>
-      <c r="CB68" s="32" t="n"/>
+      <c r="CB68" s="32" t="n">
+        <v>1</v>
+      </c>
       <c r="CC68" s="32" t="n"/>
       <c r="CD68" s="32" t="n"/>
       <c r="CE68" s="32" t="n"/>
@@ -26046,7 +26060,9 @@
       <c r="BY76" s="17" t="n"/>
       <c r="BZ76" s="17" t="n"/>
       <c r="CA76" s="17" t="n"/>
-      <c r="CB76" s="17" t="n"/>
+      <c r="CB76" s="17" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CC76" s="17" t="n"/>
       <c r="CD76" s="17" t="n"/>
       <c r="CE76" s="17" t="n"/>
@@ -31033,277 +31049,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008A7894324D7C3949B4D325554D1FC6DA" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="43dd22c4a0a55be49439aa2cba9a6031">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="be2d32d5-45e4-45f8-8cca-e731efdae529" xmlns:ns3="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="67300191881baa0ec8105967d66c0489" ns2:_="" ns3:_="">
-    <xsd:import namespace="be2d32d5-45e4-45f8-8cca-e731efdae529"/>
-    <xsd:import namespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="be2d32d5-45e4-45f8-8cca-e731efdae529" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="10" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="11" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="7ff297e6-98dc-4a77-8782-4199b303df17" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="17" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="20" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="21" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="22" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="23" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{433bb87c-b111-4230-a796-99831eb60517}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="be2d32d5-45e4-45f8-8cca-e731efdae529">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{552BB8D9-DC48-4340-BCF7-4C1B635CEC7F}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00E3C019-928C-4C37-A671-BB9F14B50437}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1440C824-587B-4F41-8DE4-A8B2A9A677C8}"/>
 </file>
</xml_diff>

<commit_message>
Update: WMiranda_2026TimeTracking.xlsx [2026-04-20 21:38 UTC]
</commit_message>
<xml_diff>
--- a/WMiranda_2026TimeTracking.xlsx
+++ b/WMiranda_2026TimeTracking.xlsx
@@ -7937,7 +7937,9 @@
         <v>0.5</v>
       </c>
       <c r="BZ11" s="17" t="n"/>
-      <c r="CA11" s="17" t="n"/>
+      <c r="CA11" s="17" t="n">
+        <v>1</v>
+      </c>
       <c r="CB11" s="17" t="n">
         <v>1.25</v>
       </c>
@@ -9661,7 +9663,9 @@
       <c r="BZ17" s="32" t="n">
         <v>1.75</v>
       </c>
-      <c r="CA17" s="32" t="n"/>
+      <c r="CA17" s="32" t="n">
+        <v>6</v>
+      </c>
       <c r="CB17" s="32" t="n">
         <v>5</v>
       </c>
@@ -14137,7 +14141,9 @@
       <c r="BZ33" s="32" t="n">
         <v>2</v>
       </c>
-      <c r="CA33" s="32" t="n"/>
+      <c r="CA33" s="32" t="n">
+        <v>1</v>
+      </c>
       <c r="CB33" s="32" t="n">
         <v>1</v>
       </c>
@@ -21814,7 +21820,9 @@
       <c r="BZ61" s="17" t="n">
         <v>1.75</v>
       </c>
-      <c r="CA61" s="17" t="n"/>
+      <c r="CA61" s="17" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CB61" s="17" t="n"/>
       <c r="CC61" s="17" t="n"/>
       <c r="CD61" s="17" t="n"/>

</xml_diff>

<commit_message>
Update: WMiranda_2026TimeTracking.xlsx [2026-04-20 21:41 UTC]
</commit_message>
<xml_diff>
--- a/WMiranda_2026TimeTracking.xlsx
+++ b/WMiranda_2026TimeTracking.xlsx
@@ -9656,7 +9656,9 @@
       <c r="BU17" s="32" t="n"/>
       <c r="BV17" s="32" t="n"/>
       <c r="BW17" s="32" t="n"/>
-      <c r="BX17" s="32" t="n"/>
+      <c r="BX17" s="32" t="n">
+        <v>1</v>
+      </c>
       <c r="BY17" s="32" t="n">
         <v>1.5</v>
       </c>
@@ -21815,7 +21817,9 @@
       <c r="BU61" s="17" t="n"/>
       <c r="BV61" s="17" t="n"/>
       <c r="BW61" s="17" t="n"/>
-      <c r="BX61" s="17" t="n"/>
+      <c r="BX61" s="17" t="n">
+        <v>1</v>
+      </c>
       <c r="BY61" s="17" t="n"/>
       <c r="BZ61" s="17" t="n">
         <v>1.75</v>
@@ -23832,7 +23836,9 @@
       <c r="BW68" s="32" t="n">
         <v>1.5</v>
       </c>
-      <c r="BX68" s="32" t="n"/>
+      <c r="BX68" s="32" t="n">
+        <v>2</v>
+      </c>
       <c r="BY68" s="32" t="n">
         <v>3.5</v>
       </c>

</xml_diff>

<commit_message>
Sync from OneDrive: WMiranda_2026TimeTracking.xlsx [2026-04-21 03:00 UTC]
</commit_message>
<xml_diff>
--- a/WMiranda_2026TimeTracking.xlsx
+++ b/WMiranda_2026TimeTracking.xlsx
@@ -31063,4 +31063,277 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008A7894324D7C3949B4D325554D1FC6DA" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="43dd22c4a0a55be49439aa2cba9a6031">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="be2d32d5-45e4-45f8-8cca-e731efdae529" xmlns:ns3="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="67300191881baa0ec8105967d66c0489" ns2:_="" ns3:_="">
+    <xsd:import namespace="be2d32d5-45e4-45f8-8cca-e731efdae529"/>
+    <xsd:import namespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="be2d32d5-45e4-45f8-8cca-e731efdae529" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="10" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="11" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="7ff297e6-98dc-4a77-8782-4199b303df17" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="17" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="20" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="21" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="22" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="23" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{433bb87c-b111-4230-a796-99831eb60517}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="be2d32d5-45e4-45f8-8cca-e731efdae529">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D7D0CBF-B5F5-488E-913C-8456B1E62D63}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1B0A511-4C07-4E5F-8F8E-84EC8F1B9FA5}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BC41CA82-9752-4F54-8660-D5BC2A163CBF}"/>
 </file>
</xml_diff>

<commit_message>
Update: WMiranda_2026TimeTracking.xlsx [2026-04-21 14:20 UTC]
</commit_message>
<xml_diff>
--- a/WMiranda_2026TimeTracking.xlsx
+++ b/WMiranda_2026TimeTracking.xlsx
@@ -9669,7 +9669,7 @@
         <v>6</v>
       </c>
       <c r="CB17" s="32" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="CC17" s="32" t="n"/>
       <c r="CD17" s="32" t="n"/>
@@ -31063,277 +31063,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008A7894324D7C3949B4D325554D1FC6DA" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="43dd22c4a0a55be49439aa2cba9a6031">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="be2d32d5-45e4-45f8-8cca-e731efdae529" xmlns:ns3="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="67300191881baa0ec8105967d66c0489" ns2:_="" ns3:_="">
-    <xsd:import namespace="be2d32d5-45e4-45f8-8cca-e731efdae529"/>
-    <xsd:import namespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="be2d32d5-45e4-45f8-8cca-e731efdae529" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="10" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="11" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="7ff297e6-98dc-4a77-8782-4199b303df17" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="17" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="20" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="21" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="22" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="23" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{433bb87c-b111-4230-a796-99831eb60517}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="be2d32d5-45e4-45f8-8cca-e731efdae529">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D7D0CBF-B5F5-488E-913C-8456B1E62D63}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1B0A511-4C07-4E5F-8F8E-84EC8F1B9FA5}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BC41CA82-9752-4F54-8660-D5BC2A163CBF}"/>
 </file>
</xml_diff>

<commit_message>
Update: WMiranda_2026TimeTracking.xlsx [2026-04-21 19:23 UTC]
</commit_message>
<xml_diff>
--- a/WMiranda_2026TimeTracking.xlsx
+++ b/WMiranda_2026TimeTracking.xlsx
@@ -7943,7 +7943,9 @@
       <c r="CB11" s="17" t="n">
         <v>1.25</v>
       </c>
-      <c r="CC11" s="17" t="n"/>
+      <c r="CC11" s="17" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CD11" s="17" t="n"/>
       <c r="CE11" s="17" t="n"/>
       <c r="CF11" s="17" t="n"/>
@@ -8217,7 +8219,9 @@
       <c r="CB12" s="17" t="n">
         <v>0.25</v>
       </c>
-      <c r="CC12" s="17" t="n"/>
+      <c r="CC12" s="17" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CD12" s="17" t="n"/>
       <c r="CE12" s="17" t="n"/>
       <c r="CF12" s="17" t="n"/>
@@ -9671,7 +9675,9 @@
       <c r="CB17" s="32" t="n">
         <v>6</v>
       </c>
-      <c r="CC17" s="32" t="n"/>
+      <c r="CC17" s="32" t="n">
+        <v>3.5</v>
+      </c>
       <c r="CD17" s="32" t="n"/>
       <c r="CE17" s="32" t="n"/>
       <c r="CF17" s="32" t="n"/>
@@ -14149,7 +14155,9 @@
       <c r="CB33" s="32" t="n">
         <v>1</v>
       </c>
-      <c r="CC33" s="32" t="n"/>
+      <c r="CC33" s="32" t="n">
+        <v>1.25</v>
+      </c>
       <c r="CD33" s="32" t="n"/>
       <c r="CE33" s="32" t="n"/>
       <c r="CF33" s="32" t="n"/>
@@ -23511,7 +23519,9 @@
       <c r="BZ67" s="32" t="n"/>
       <c r="CA67" s="32" t="n"/>
       <c r="CB67" s="32" t="n"/>
-      <c r="CC67" s="32" t="n"/>
+      <c r="CC67" s="32" t="n">
+        <v>1.25</v>
+      </c>
       <c r="CD67" s="32" t="n"/>
       <c r="CE67" s="32" t="n"/>
       <c r="CF67" s="32" t="n"/>
@@ -23849,7 +23859,9 @@
       <c r="CB68" s="32" t="n">
         <v>1</v>
       </c>
-      <c r="CC68" s="32" t="n"/>
+      <c r="CC68" s="32" t="n">
+        <v>1.75</v>
+      </c>
       <c r="CD68" s="32" t="n"/>
       <c r="CE68" s="32" t="n"/>
       <c r="CF68" s="32" t="n"/>

</xml_diff>

<commit_message>
Update: WMiranda_2026TimeTracking.xlsx [2026-04-22 20:39 UTC]
</commit_message>
<xml_diff>
--- a/WMiranda_2026TimeTracking.xlsx
+++ b/WMiranda_2026TimeTracking.xlsx
@@ -7946,7 +7946,9 @@
       <c r="CC11" s="17" t="n">
         <v>1.5</v>
       </c>
-      <c r="CD11" s="17" t="n"/>
+      <c r="CD11" s="17" t="n">
+        <v>1</v>
+      </c>
       <c r="CE11" s="17" t="n"/>
       <c r="CF11" s="17" t="n"/>
       <c r="CG11" s="17" t="n"/>
@@ -23522,7 +23524,9 @@
       <c r="CC67" s="32" t="n">
         <v>1.25</v>
       </c>
-      <c r="CD67" s="32" t="n"/>
+      <c r="CD67" s="32" t="n">
+        <v>2</v>
+      </c>
       <c r="CE67" s="32" t="n"/>
       <c r="CF67" s="32" t="n"/>
       <c r="CG67" s="32" t="n"/>
@@ -23862,7 +23866,9 @@
       <c r="CC68" s="32" t="n">
         <v>1.75</v>
       </c>
-      <c r="CD68" s="32" t="n"/>
+      <c r="CD68" s="32" t="n">
+        <v>5</v>
+      </c>
       <c r="CE68" s="32" t="n"/>
       <c r="CF68" s="32" t="n"/>
       <c r="CG68" s="32" t="n"/>
@@ -26090,7 +26096,9 @@
         <v>0.25</v>
       </c>
       <c r="CC76" s="17" t="n"/>
-      <c r="CD76" s="17" t="n"/>
+      <c r="CD76" s="17" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CE76" s="17" t="n"/>
       <c r="CF76" s="17" t="n"/>
       <c r="CG76" s="17" t="n"/>

</xml_diff>

<commit_message>
Update: WMiranda_2026TimeTracking.xlsx [2026-04-23 20:40 UTC]
</commit_message>
<xml_diff>
--- a/WMiranda_2026TimeTracking.xlsx
+++ b/WMiranda_2026TimeTracking.xlsx
@@ -7949,7 +7949,9 @@
       <c r="CD11" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="CE11" s="17" t="n"/>
+      <c r="CE11" s="17" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CF11" s="17" t="n"/>
       <c r="CG11" s="17" t="n"/>
       <c r="CH11" s="17" t="n"/>
@@ -9681,7 +9683,9 @@
         <v>3.5</v>
       </c>
       <c r="CD17" s="32" t="n"/>
-      <c r="CE17" s="32" t="n"/>
+      <c r="CE17" s="32" t="n">
+        <v>1.25</v>
+      </c>
       <c r="CF17" s="32" t="n"/>
       <c r="CG17" s="32" t="n"/>
       <c r="CH17" s="32" t="n"/>
@@ -18824,7 +18828,9 @@
       </c>
       <c r="CC50" s="17" t="n"/>
       <c r="CD50" s="17" t="n"/>
-      <c r="CE50" s="17" t="n"/>
+      <c r="CE50" s="17" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CF50" s="17" t="n"/>
       <c r="CG50" s="17" t="n"/>
       <c r="CH50" s="17" t="n"/>
@@ -22937,7 +22943,9 @@
       <c r="CB65" s="20" t="n"/>
       <c r="CC65" s="20" t="n"/>
       <c r="CD65" s="20" t="n"/>
-      <c r="CE65" s="20" t="n"/>
+      <c r="CE65" s="20" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CF65" s="20" t="n"/>
       <c r="CG65" s="20" t="n"/>
       <c r="CH65" s="20" t="n"/>
@@ -23527,7 +23535,9 @@
       <c r="CD67" s="32" t="n">
         <v>2</v>
       </c>
-      <c r="CE67" s="32" t="n"/>
+      <c r="CE67" s="32" t="n">
+        <v>2</v>
+      </c>
       <c r="CF67" s="32" t="n"/>
       <c r="CG67" s="32" t="n"/>
       <c r="CH67" s="32" t="n"/>
@@ -23869,7 +23879,9 @@
       <c r="CD68" s="32" t="n">
         <v>5</v>
       </c>
-      <c r="CE68" s="32" t="n"/>
+      <c r="CE68" s="32" t="n">
+        <v>2</v>
+      </c>
       <c r="CF68" s="32" t="n"/>
       <c r="CG68" s="32" t="n"/>
       <c r="CH68" s="32" t="n"/>
@@ -27231,7 +27243,9 @@
       <c r="CB80" s="17" t="n"/>
       <c r="CC80" s="17" t="n"/>
       <c r="CD80" s="17" t="n"/>
-      <c r="CE80" s="17" t="n"/>
+      <c r="CE80" s="17" t="n">
+        <v>1</v>
+      </c>
       <c r="CF80" s="17" t="n"/>
       <c r="CG80" s="17" t="n"/>
       <c r="CH80" s="17" t="n"/>

</xml_diff>

<commit_message>
Update: WMiranda_2026TimeTracking.xlsx [2026-04-24 19:44 UTC]
</commit_message>
<xml_diff>
--- a/WMiranda_2026TimeTracking.xlsx
+++ b/WMiranda_2026TimeTracking.xlsx
@@ -9686,7 +9686,9 @@
       <c r="CE17" s="32" t="n">
         <v>1.25</v>
       </c>
-      <c r="CF17" s="32" t="n"/>
+      <c r="CF17" s="32" t="n">
+        <v>2.5</v>
+      </c>
       <c r="CG17" s="32" t="n"/>
       <c r="CH17" s="32" t="n"/>
       <c r="CI17" s="32" t="n"/>
@@ -14166,7 +14168,9 @@
       </c>
       <c r="CD33" s="32" t="n"/>
       <c r="CE33" s="32" t="n"/>
-      <c r="CF33" s="32" t="n"/>
+      <c r="CF33" s="32" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CG33" s="32" t="n"/>
       <c r="CH33" s="32" t="n"/>
       <c r="CI33" s="32" t="n"/>
@@ -19103,7 +19107,9 @@
       <c r="CC51" s="17" t="n"/>
       <c r="CD51" s="17" t="n"/>
       <c r="CE51" s="17" t="n"/>
-      <c r="CF51" s="17" t="n"/>
+      <c r="CF51" s="17" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CG51" s="17" t="n"/>
       <c r="CH51" s="17" t="n"/>
       <c r="CI51" s="17" t="n"/>
@@ -23538,7 +23544,9 @@
       <c r="CE67" s="32" t="n">
         <v>2</v>
       </c>
-      <c r="CF67" s="32" t="n"/>
+      <c r="CF67" s="32" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CG67" s="32" t="n"/>
       <c r="CH67" s="32" t="n"/>
       <c r="CI67" s="32" t="n"/>
@@ -23882,7 +23890,9 @@
       <c r="CE68" s="32" t="n">
         <v>2</v>
       </c>
-      <c r="CF68" s="32" t="n"/>
+      <c r="CF68" s="32" t="n">
+        <v>2.5</v>
+      </c>
       <c r="CG68" s="32" t="n"/>
       <c r="CH68" s="32" t="n"/>
       <c r="CI68" s="32" t="n"/>
@@ -26404,7 +26414,9 @@
       <c r="CC77" s="17" t="n"/>
       <c r="CD77" s="17" t="n"/>
       <c r="CE77" s="17" t="n"/>
-      <c r="CF77" s="17" t="n"/>
+      <c r="CF77" s="17" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CG77" s="17" t="n"/>
       <c r="CH77" s="17" t="n"/>
       <c r="CI77" s="17" t="n"/>

</xml_diff>

<commit_message>
Update: WMiranda_2026TimeTracking.xlsx [2026-04-27 19:48 UTC]
</commit_message>
<xml_diff>
--- a/WMiranda_2026TimeTracking.xlsx
+++ b/WMiranda_2026TimeTracking.xlsx
@@ -7953,7 +7953,9 @@
         <v>0.25</v>
       </c>
       <c r="CF11" s="17" t="n"/>
-      <c r="CG11" s="17" t="n"/>
+      <c r="CG11" s="17" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CH11" s="17" t="n"/>
       <c r="CI11" s="17" t="n"/>
       <c r="CJ11" s="18" t="n"/>
@@ -9689,7 +9691,9 @@
       <c r="CF17" s="32" t="n">
         <v>2.5</v>
       </c>
-      <c r="CG17" s="32" t="n"/>
+      <c r="CG17" s="32" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CH17" s="32" t="n"/>
       <c r="CI17" s="32" t="n"/>
       <c r="CJ17" s="33" t="n"/>
@@ -23547,7 +23551,9 @@
       <c r="CF67" s="32" t="n">
         <v>0.5</v>
       </c>
-      <c r="CG67" s="32" t="n"/>
+      <c r="CG67" s="32" t="n">
+        <v>1</v>
+      </c>
       <c r="CH67" s="32" t="n"/>
       <c r="CI67" s="32" t="n"/>
       <c r="CJ67" s="33" t="n"/>
@@ -23893,7 +23899,9 @@
       <c r="CF68" s="32" t="n">
         <v>2.5</v>
       </c>
-      <c r="CG68" s="32" t="n"/>
+      <c r="CG68" s="32" t="n">
+        <v>5</v>
+      </c>
       <c r="CH68" s="32" t="n"/>
       <c r="CI68" s="32" t="n"/>
       <c r="CJ68" s="33" t="n"/>

</xml_diff>

<commit_message>
Update: WMiranda_2026TimeTracking.xlsx [2026-04-28 20:50 UTC]
</commit_message>
<xml_diff>
--- a/WMiranda_2026TimeTracking.xlsx
+++ b/WMiranda_2026TimeTracking.xlsx
@@ -9694,7 +9694,9 @@
       <c r="CG17" s="32" t="n">
         <v>0.5</v>
       </c>
-      <c r="CH17" s="32" t="n"/>
+      <c r="CH17" s="32" t="n">
+        <v>2.25</v>
+      </c>
       <c r="CI17" s="32" t="n"/>
       <c r="CJ17" s="33" t="n"/>
       <c r="CK17" s="32" t="n"/>
@@ -10816,7 +10818,9 @@
       <c r="CE21" s="17" t="n"/>
       <c r="CF21" s="17" t="n"/>
       <c r="CG21" s="17" t="n"/>
-      <c r="CH21" s="17" t="n"/>
+      <c r="CH21" s="17" t="n">
+        <v>0.75</v>
+      </c>
       <c r="CI21" s="17" t="n"/>
       <c r="CJ21" s="18" t="n"/>
       <c r="CK21" s="17" t="n"/>
@@ -23554,7 +23558,9 @@
       <c r="CG67" s="32" t="n">
         <v>1</v>
       </c>
-      <c r="CH67" s="32" t="n"/>
+      <c r="CH67" s="32" t="n">
+        <v>1</v>
+      </c>
       <c r="CI67" s="32" t="n"/>
       <c r="CJ67" s="33" t="n"/>
       <c r="CK67" s="32" t="n"/>
@@ -23902,7 +23908,9 @@
       <c r="CG68" s="32" t="n">
         <v>5</v>
       </c>
-      <c r="CH68" s="32" t="n"/>
+      <c r="CH68" s="32" t="n">
+        <v>4.25</v>
+      </c>
       <c r="CI68" s="32" t="n"/>
       <c r="CJ68" s="33" t="n"/>
       <c r="CK68" s="32" t="n"/>

</xml_diff>

<commit_message>
Update: WMiranda_2026TimeTracking.xlsx [2026-04-29 19:55 UTC]
</commit_message>
<xml_diff>
--- a/WMiranda_2026TimeTracking.xlsx
+++ b/WMiranda_2026TimeTracking.xlsx
@@ -7359,7 +7359,9 @@
       <c r="CF9" s="32" t="n"/>
       <c r="CG9" s="32" t="n"/>
       <c r="CH9" s="32" t="n"/>
-      <c r="CI9" s="32" t="n"/>
+      <c r="CI9" s="32" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CJ9" s="33" t="n"/>
       <c r="CK9" s="32" t="n"/>
       <c r="CL9" s="32" t="n"/>
@@ -7957,7 +7959,9 @@
         <v>1.5</v>
       </c>
       <c r="CH11" s="17" t="n"/>
-      <c r="CI11" s="17" t="n"/>
+      <c r="CI11" s="17" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CJ11" s="18" t="n"/>
       <c r="CK11" s="17" t="n"/>
       <c r="CL11" s="17" t="n"/>
@@ -14181,7 +14185,9 @@
       </c>
       <c r="CG33" s="32" t="n"/>
       <c r="CH33" s="32" t="n"/>
-      <c r="CI33" s="32" t="n"/>
+      <c r="CI33" s="32" t="n">
+        <v>2</v>
+      </c>
       <c r="CJ33" s="33" t="n"/>
       <c r="CK33" s="32" t="n"/>
       <c r="CL33" s="32" t="n"/>
@@ -17470,7 +17476,9 @@
       <c r="CF45" s="17" t="n"/>
       <c r="CG45" s="17" t="n"/>
       <c r="CH45" s="17" t="n"/>
-      <c r="CI45" s="17" t="n"/>
+      <c r="CI45" s="17" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CJ45" s="18" t="n"/>
       <c r="CK45" s="17" t="n"/>
       <c r="CL45" s="17" t="n"/>
@@ -23911,7 +23919,9 @@
       <c r="CH68" s="32" t="n">
         <v>4.25</v>
       </c>
-      <c r="CI68" s="32" t="n"/>
+      <c r="CI68" s="32" t="n">
+        <v>2.5</v>
+      </c>
       <c r="CJ68" s="33" t="n"/>
       <c r="CK68" s="32" t="n"/>
       <c r="CL68" s="32" t="n"/>
@@ -24183,7 +24193,9 @@
       <c r="CF69" s="17" t="n"/>
       <c r="CG69" s="17" t="n"/>
       <c r="CH69" s="17" t="n"/>
-      <c r="CI69" s="17" t="n"/>
+      <c r="CI69" s="17" t="n">
+        <v>1</v>
+      </c>
       <c r="CJ69" s="18" t="n"/>
       <c r="CK69" s="17" t="n"/>
       <c r="CL69" s="17" t="n"/>

</xml_diff>

<commit_message>
Update: WMiranda_2026TimeTracking.xlsx [2026-04-30 10:51 UTC]
</commit_message>
<xml_diff>
--- a/WMiranda_2026TimeTracking.xlsx
+++ b/WMiranda_2026TimeTracking.xlsx
@@ -14188,7 +14188,9 @@
       <c r="CI33" s="32" t="n">
         <v>2</v>
       </c>
-      <c r="CJ33" s="33" t="n"/>
+      <c r="CJ33" s="33" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CK33" s="32" t="n"/>
       <c r="CL33" s="32" t="n"/>
       <c r="CM33" s="32" t="n"/>
@@ -23922,7 +23924,9 @@
       <c r="CI68" s="32" t="n">
         <v>3</v>
       </c>
-      <c r="CJ68" s="33" t="n"/>
+      <c r="CJ68" s="33" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CK68" s="32" t="n"/>
       <c r="CL68" s="32" t="n"/>
       <c r="CM68" s="32" t="n"/>

</xml_diff>

<commit_message>
Update: WMiranda_2026TimeTracking.xlsx [2026-04-30 20:44 UTC]
</commit_message>
<xml_diff>
--- a/WMiranda_2026TimeTracking.xlsx
+++ b/WMiranda_2026TimeTracking.xlsx
@@ -17481,7 +17481,9 @@
       <c r="CI45" s="17" t="n">
         <v>0.5</v>
       </c>
-      <c r="CJ45" s="18" t="n"/>
+      <c r="CJ45" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CK45" s="17" t="n"/>
       <c r="CL45" s="17" t="n"/>
       <c r="CM45" s="17" t="n"/>
@@ -22974,7 +22976,9 @@
       <c r="CG65" s="20" t="n"/>
       <c r="CH65" s="20" t="n"/>
       <c r="CI65" s="20" t="n"/>
-      <c r="CJ65" s="22" t="n"/>
+      <c r="CJ65" s="22" t="n">
+        <v>0.75</v>
+      </c>
       <c r="CK65" s="20" t="n"/>
       <c r="CL65" s="20" t="n"/>
       <c r="CM65" s="20" t="n"/>
@@ -23572,7 +23576,9 @@
         <v>1</v>
       </c>
       <c r="CI67" s="32" t="n"/>
-      <c r="CJ67" s="33" t="n"/>
+      <c r="CJ67" s="33" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CK67" s="32" t="n"/>
       <c r="CL67" s="32" t="n"/>
       <c r="CM67" s="32" t="n"/>
@@ -23925,7 +23931,7 @@
         <v>3</v>
       </c>
       <c r="CJ68" s="33" t="n">
-        <v>0.5</v>
+        <v>3</v>
       </c>
       <c r="CK68" s="32" t="n"/>
       <c r="CL68" s="32" t="n"/>
@@ -27294,7 +27300,9 @@
       <c r="CG80" s="17" t="n"/>
       <c r="CH80" s="17" t="n"/>
       <c r="CI80" s="17" t="n"/>
-      <c r="CJ80" s="18" t="n"/>
+      <c r="CJ80" s="18" t="n">
+        <v>3.5</v>
+      </c>
       <c r="CK80" s="17" t="n"/>
       <c r="CL80" s="17" t="n"/>
       <c r="CM80" s="17" t="n"/>

</xml_diff>

<commit_message>
Update: WMiranda_2026TimeTracking.xlsx [2026-05-01 20:32 UTC]
</commit_message>
<xml_diff>
--- a/WMiranda_2026TimeTracking.xlsx
+++ b/WMiranda_2026TimeTracking.xlsx
@@ -7963,7 +7963,9 @@
         <v>0.5</v>
       </c>
       <c r="CJ11" s="18" t="n"/>
-      <c r="CK11" s="17" t="n"/>
+      <c r="CK11" s="17" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CL11" s="17" t="n"/>
       <c r="CM11" s="17" t="n"/>
       <c r="CN11" s="17" t="n"/>
@@ -9703,7 +9705,9 @@
       </c>
       <c r="CI17" s="32" t="n"/>
       <c r="CJ17" s="33" t="n"/>
-      <c r="CK17" s="32" t="n"/>
+      <c r="CK17" s="32" t="n">
+        <v>1</v>
+      </c>
       <c r="CL17" s="32" t="n"/>
       <c r="CM17" s="32" t="n"/>
       <c r="CN17" s="32" t="n"/>
@@ -14191,7 +14195,9 @@
       <c r="CJ33" s="33" t="n">
         <v>0.5</v>
       </c>
-      <c r="CK33" s="32" t="n"/>
+      <c r="CK33" s="32" t="n">
+        <v>2.5</v>
+      </c>
       <c r="CL33" s="32" t="n"/>
       <c r="CM33" s="32" t="n"/>
       <c r="CN33" s="32" t="n"/>
@@ -20243,7 +20249,9 @@
       <c r="CH55" s="32" t="n"/>
       <c r="CI55" s="32" t="n"/>
       <c r="CJ55" s="33" t="n"/>
-      <c r="CK55" s="32" t="n"/>
+      <c r="CK55" s="32" t="n">
+        <v>0.75</v>
+      </c>
       <c r="CL55" s="32" t="n"/>
       <c r="CM55" s="32" t="n"/>
       <c r="CN55" s="32" t="n"/>
@@ -23933,7 +23941,9 @@
       <c r="CJ68" s="33" t="n">
         <v>3</v>
       </c>
-      <c r="CK68" s="32" t="n"/>
+      <c r="CK68" s="32" t="n">
+        <v>3.5</v>
+      </c>
       <c r="CL68" s="32" t="n"/>
       <c r="CM68" s="32" t="n"/>
       <c r="CN68" s="32" t="n"/>

</xml_diff>

<commit_message>
Update: WMiranda_2026TimeTracking.xlsx [2026-05-01 20:33 UTC]
</commit_message>
<xml_diff>
--- a/WMiranda_2026TimeTracking.xlsx
+++ b/WMiranda_2026TimeTracking.xlsx
@@ -13022,7 +13022,9 @@
       <c r="CH29" s="17" t="n"/>
       <c r="CI29" s="17" t="n"/>
       <c r="CJ29" s="18" t="n"/>
-      <c r="CK29" s="17" t="n"/>
+      <c r="CK29" s="17" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CL29" s="17" t="n"/>
       <c r="CM29" s="17" t="n"/>
       <c r="CN29" s="17" t="n"/>

</xml_diff>

<commit_message>
Update: WMiranda_2026TimeTracking.xlsx [2026-05-04 17:48 UTC]
</commit_message>
<xml_diff>
--- a/WMiranda_2026TimeTracking.xlsx
+++ b/WMiranda_2026TimeTracking.xlsx
@@ -23946,7 +23946,9 @@
       <c r="CK68" s="32" t="n">
         <v>3.5</v>
       </c>
-      <c r="CL68" s="32" t="n"/>
+      <c r="CL68" s="32" t="n">
+        <v>12</v>
+      </c>
       <c r="CM68" s="32" t="n"/>
       <c r="CN68" s="32" t="n"/>
       <c r="CO68" s="32" t="n"/>

</xml_diff>

<commit_message>
Update: WMiranda_2026TimeTracking.xlsx [2026-05-05 20:42 UTC]
</commit_message>
<xml_diff>
--- a/WMiranda_2026TimeTracking.xlsx
+++ b/WMiranda_2026TimeTracking.xlsx
@@ -7365,7 +7365,9 @@
       <c r="CJ9" s="33" t="n"/>
       <c r="CK9" s="32" t="n"/>
       <c r="CL9" s="32" t="n"/>
-      <c r="CM9" s="32" t="n"/>
+      <c r="CM9" s="32" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CN9" s="32" t="n"/>
       <c r="CO9" s="32" t="n"/>
       <c r="CP9" s="32" t="n"/>
@@ -9709,7 +9711,9 @@
         <v>1</v>
       </c>
       <c r="CL17" s="32" t="n"/>
-      <c r="CM17" s="32" t="n"/>
+      <c r="CM17" s="32" t="n">
+        <v>2</v>
+      </c>
       <c r="CN17" s="32" t="n"/>
       <c r="CO17" s="32" t="n"/>
       <c r="CP17" s="32" t="n"/>
@@ -20255,7 +20259,9 @@
         <v>0.75</v>
       </c>
       <c r="CL55" s="32" t="n"/>
-      <c r="CM55" s="32" t="n"/>
+      <c r="CM55" s="32" t="n">
+        <v>1</v>
+      </c>
       <c r="CN55" s="32" t="n"/>
       <c r="CO55" s="32" t="n"/>
       <c r="CP55" s="32" t="n"/>
@@ -23949,7 +23955,9 @@
       <c r="CL68" s="32" t="n">
         <v>12</v>
       </c>
-      <c r="CM68" s="32" t="n"/>
+      <c r="CM68" s="32" t="n">
+        <v>5.5</v>
+      </c>
       <c r="CN68" s="32" t="n"/>
       <c r="CO68" s="32" t="n"/>
       <c r="CP68" s="32" t="n"/>

</xml_diff>

<commit_message>
Update: WMiranda_2026TimeTracking.xlsx [2026-05-06 20:37 UTC]
</commit_message>
<xml_diff>
--- a/WMiranda_2026TimeTracking.xlsx
+++ b/WMiranda_2026TimeTracking.xlsx
@@ -14206,7 +14206,9 @@
       </c>
       <c r="CL33" s="32" t="n"/>
       <c r="CM33" s="32" t="n"/>
-      <c r="CN33" s="32" t="n"/>
+      <c r="CN33" s="32" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CO33" s="32" t="n"/>
       <c r="CP33" s="32" t="n"/>
       <c r="CQ33" s="32" t="n"/>
@@ -23958,7 +23960,9 @@
       <c r="CM68" s="32" t="n">
         <v>5.5</v>
       </c>
-      <c r="CN68" s="32" t="n"/>
+      <c r="CN68" s="32" t="n">
+        <v>8</v>
+      </c>
       <c r="CO68" s="32" t="n"/>
       <c r="CP68" s="32" t="n"/>
       <c r="CQ68" s="32" t="n"/>

</xml_diff>

<commit_message>
Update: WMiranda_2026TimeTracking.xlsx [2026-05-13 17:28 UTC]
</commit_message>
<xml_diff>
--- a/WMiranda_2026TimeTracking.xlsx
+++ b/WMiranda_2026TimeTracking.xlsx
@@ -9715,7 +9715,9 @@
         <v>2</v>
       </c>
       <c r="CN17" s="32" t="n"/>
-      <c r="CO17" s="32" t="n"/>
+      <c r="CO17" s="32" t="n">
+        <v>2</v>
+      </c>
       <c r="CP17" s="32" t="n"/>
       <c r="CQ17" s="32" t="n"/>
       <c r="CR17" s="32" t="n"/>
@@ -23963,7 +23965,9 @@
       <c r="CN68" s="32" t="n">
         <v>8</v>
       </c>
-      <c r="CO68" s="32" t="n"/>
+      <c r="CO68" s="32" t="n">
+        <v>7</v>
+      </c>
       <c r="CP68" s="32" t="n"/>
       <c r="CQ68" s="32" t="n"/>
       <c r="CR68" s="32" t="n"/>

</xml_diff>

<commit_message>
Update: WMiranda_2026TimeTracking.xlsx [2026-05-13 17:31 UTC]
</commit_message>
<xml_diff>
--- a/WMiranda_2026TimeTracking.xlsx
+++ b/WMiranda_2026TimeTracking.xlsx
@@ -9718,7 +9718,9 @@
       <c r="CO17" s="32" t="n">
         <v>2</v>
       </c>
-      <c r="CP17" s="32" t="n"/>
+      <c r="CP17" s="32" t="n">
+        <v>1</v>
+      </c>
       <c r="CQ17" s="32" t="n"/>
       <c r="CR17" s="32" t="n"/>
       <c r="CS17" s="32" t="n"/>
@@ -10006,7 +10008,9 @@
       <c r="CM18" s="17" t="n"/>
       <c r="CN18" s="17" t="n"/>
       <c r="CO18" s="17" t="n"/>
-      <c r="CP18" s="17" t="n"/>
+      <c r="CP18" s="17" t="n">
+        <v>2</v>
+      </c>
       <c r="CQ18" s="17" t="n"/>
       <c r="CR18" s="17" t="n"/>
       <c r="CS18" s="17" t="n"/>
@@ -14212,7 +14216,9 @@
         <v>1.5</v>
       </c>
       <c r="CO33" s="32" t="n"/>
-      <c r="CP33" s="32" t="n"/>
+      <c r="CP33" s="32" t="n">
+        <v>4</v>
+      </c>
       <c r="CQ33" s="32" t="n"/>
       <c r="CR33" s="32" t="n"/>
       <c r="CS33" s="32" t="n"/>
@@ -23968,7 +23974,9 @@
       <c r="CO68" s="32" t="n">
         <v>7</v>
       </c>
-      <c r="CP68" s="32" t="n"/>
+      <c r="CP68" s="32" t="n">
+        <v>4</v>
+      </c>
       <c r="CQ68" s="32" t="n"/>
       <c r="CR68" s="32" t="n"/>
       <c r="CS68" s="32" t="n"/>

</xml_diff>

<commit_message>
Update: WMiranda_2026TimeTracking.xlsx [2026-05-13 17:33 UTC]
</commit_message>
<xml_diff>
--- a/WMiranda_2026TimeTracking.xlsx
+++ b/WMiranda_2026TimeTracking.xlsx
@@ -7973,7 +7973,9 @@
       <c r="CN11" s="17" t="n"/>
       <c r="CO11" s="17" t="n"/>
       <c r="CP11" s="17" t="n"/>
-      <c r="CQ11" s="17" t="n"/>
+      <c r="CQ11" s="17" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CR11" s="17" t="n"/>
       <c r="CS11" s="17" t="n"/>
       <c r="CT11" s="17" t="n"/>
@@ -9721,7 +9723,9 @@
       <c r="CP17" s="32" t="n">
         <v>1</v>
       </c>
-      <c r="CQ17" s="32" t="n"/>
+      <c r="CQ17" s="32" t="n">
+        <v>1.75</v>
+      </c>
       <c r="CR17" s="32" t="n"/>
       <c r="CS17" s="32" t="n"/>
       <c r="CT17" s="32" t="n"/>
@@ -14219,7 +14223,9 @@
       <c r="CP33" s="32" t="n">
         <v>4</v>
       </c>
-      <c r="CQ33" s="32" t="n"/>
+      <c r="CQ33" s="32" t="n">
+        <v>1.25</v>
+      </c>
       <c r="CR33" s="32" t="n"/>
       <c r="CS33" s="32" t="n"/>
       <c r="CT33" s="32" t="n"/>
@@ -18888,7 +18894,9 @@
       <c r="CN50" s="17" t="n"/>
       <c r="CO50" s="17" t="n"/>
       <c r="CP50" s="17" t="n"/>
-      <c r="CQ50" s="17" t="n"/>
+      <c r="CQ50" s="17" t="n">
+        <v>1</v>
+      </c>
       <c r="CR50" s="17" t="n"/>
       <c r="CS50" s="17" t="n"/>
       <c r="CT50" s="17" t="n"/>
@@ -23611,7 +23619,9 @@
       <c r="CN67" s="32" t="n"/>
       <c r="CO67" s="32" t="n"/>
       <c r="CP67" s="32" t="n"/>
-      <c r="CQ67" s="32" t="n"/>
+      <c r="CQ67" s="32" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CR67" s="32" t="n"/>
       <c r="CS67" s="32" t="n"/>
       <c r="CT67" s="32" t="n"/>
@@ -23977,7 +23987,9 @@
       <c r="CP68" s="32" t="n">
         <v>4</v>
       </c>
-      <c r="CQ68" s="32" t="n"/>
+      <c r="CQ68" s="32" t="n">
+        <v>2</v>
+      </c>
       <c r="CR68" s="32" t="n"/>
       <c r="CS68" s="32" t="n"/>
       <c r="CT68" s="32" t="n"/>

</xml_diff>

<commit_message>
Update: WMiranda_2026TimeTracking.xlsx [2026-05-13 17:37 UTC]
</commit_message>
<xml_diff>
--- a/WMiranda_2026TimeTracking.xlsx
+++ b/WMiranda_2026TimeTracking.xlsx
@@ -7976,7 +7976,9 @@
       <c r="CQ11" s="17" t="n">
         <v>1.5</v>
       </c>
-      <c r="CR11" s="17" t="n"/>
+      <c r="CR11" s="17" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CS11" s="17" t="n"/>
       <c r="CT11" s="17" t="n"/>
       <c r="CU11" s="17" t="n"/>
@@ -9726,7 +9728,9 @@
       <c r="CQ17" s="32" t="n">
         <v>1.75</v>
       </c>
-      <c r="CR17" s="32" t="n"/>
+      <c r="CR17" s="32" t="n">
+        <v>2.75</v>
+      </c>
       <c r="CS17" s="32" t="n"/>
       <c r="CT17" s="32" t="n"/>
       <c r="CU17" s="32" t="n"/>
@@ -14226,7 +14230,9 @@
       <c r="CQ33" s="32" t="n">
         <v>1.25</v>
       </c>
-      <c r="CR33" s="32" t="n"/>
+      <c r="CR33" s="32" t="n">
+        <v>1</v>
+      </c>
       <c r="CS33" s="32" t="n"/>
       <c r="CT33" s="32" t="n"/>
       <c r="CU33" s="32" t="n"/>
@@ -16957,7 +16963,9 @@
       <c r="CO43" s="17" t="n"/>
       <c r="CP43" s="17" t="n"/>
       <c r="CQ43" s="17" t="n"/>
-      <c r="CR43" s="17" t="n"/>
+      <c r="CR43" s="17" t="n">
+        <v>1</v>
+      </c>
       <c r="CS43" s="17" t="n"/>
       <c r="CT43" s="17" t="n"/>
       <c r="CU43" s="17" t="n"/>
@@ -23622,7 +23630,9 @@
       <c r="CQ67" s="32" t="n">
         <v>1.5</v>
       </c>
-      <c r="CR67" s="32" t="n"/>
+      <c r="CR67" s="32" t="n">
+        <v>1.75</v>
+      </c>
       <c r="CS67" s="32" t="n"/>
       <c r="CT67" s="32" t="n"/>
       <c r="CU67" s="32" t="n"/>
@@ -23990,7 +24000,9 @@
       <c r="CQ68" s="32" t="n">
         <v>2</v>
       </c>
-      <c r="CR68" s="32" t="n"/>
+      <c r="CR68" s="32" t="n">
+        <v>1</v>
+      </c>
       <c r="CS68" s="32" t="n"/>
       <c r="CT68" s="32" t="n"/>
       <c r="CU68" s="32" t="n"/>

</xml_diff>

<commit_message>
Update: WMiranda_2026TimeTracking.xlsx [2026-05-14 16:38 UTC]
</commit_message>
<xml_diff>
--- a/WMiranda_2026TimeTracking.xlsx
+++ b/WMiranda_2026TimeTracking.xlsx
@@ -7374,7 +7374,9 @@
       <c r="CQ9" s="32" t="n"/>
       <c r="CR9" s="32" t="n"/>
       <c r="CS9" s="32" t="n"/>
-      <c r="CT9" s="32" t="n"/>
+      <c r="CT9" s="32" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CU9" s="32" t="n"/>
       <c r="CV9" s="32" t="n"/>
       <c r="CW9" s="32" t="n"/>
@@ -9732,7 +9734,9 @@
         <v>2.75</v>
       </c>
       <c r="CS17" s="32" t="n"/>
-      <c r="CT17" s="32" t="n"/>
+      <c r="CT17" s="32" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CU17" s="32" t="n"/>
       <c r="CV17" s="32" t="n"/>
       <c r="CW17" s="32" t="n"/>
@@ -14234,7 +14238,9 @@
         <v>1</v>
       </c>
       <c r="CS33" s="32" t="n"/>
-      <c r="CT33" s="32" t="n"/>
+      <c r="CT33" s="32" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CU33" s="32" t="n"/>
       <c r="CV33" s="32" t="n"/>
       <c r="CW33" s="32" t="n"/>
@@ -16967,7 +16973,9 @@
         <v>1</v>
       </c>
       <c r="CS43" s="17" t="n"/>
-      <c r="CT43" s="17" t="n"/>
+      <c r="CT43" s="17" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CU43" s="17" t="n"/>
       <c r="CV43" s="17" t="n"/>
       <c r="CW43" s="17" t="n"/>
@@ -23634,7 +23642,9 @@
         <v>1.75</v>
       </c>
       <c r="CS67" s="32" t="n"/>
-      <c r="CT67" s="32" t="n"/>
+      <c r="CT67" s="32" t="n">
+        <v>2</v>
+      </c>
       <c r="CU67" s="32" t="n"/>
       <c r="CV67" s="32" t="n"/>
       <c r="CW67" s="32" t="n"/>
@@ -24004,7 +24014,9 @@
         <v>1</v>
       </c>
       <c r="CS68" s="32" t="n"/>
-      <c r="CT68" s="32" t="n"/>
+      <c r="CT68" s="32" t="n">
+        <v>2</v>
+      </c>
       <c r="CU68" s="32" t="n"/>
       <c r="CV68" s="32" t="n"/>
       <c r="CW68" s="32" t="n"/>

</xml_diff>

<commit_message>
Update: WMiranda_2026TimeTracking.xlsx [2026-05-14 16:39 UTC]
</commit_message>
<xml_diff>
--- a/WMiranda_2026TimeTracking.xlsx
+++ b/WMiranda_2026TimeTracking.xlsx
@@ -27967,7 +27967,9 @@
       <c r="CR82" s="17" t="n"/>
       <c r="CS82" s="17" t="n"/>
       <c r="CT82" s="17" t="n"/>
-      <c r="CU82" s="17" t="n"/>
+      <c r="CU82" s="17" t="n">
+        <v>8</v>
+      </c>
       <c r="CV82" s="17" t="n"/>
       <c r="CW82" s="17" t="n"/>
       <c r="CX82" s="17" t="n"/>

</xml_diff>

<commit_message>
Update: WMiranda_2026TimeTracking.xlsx [2026-05-14 16:41 UTC]
</commit_message>
<xml_diff>
--- a/WMiranda_2026TimeTracking.xlsx
+++ b/WMiranda_2026TimeTracking.xlsx
@@ -7373,7 +7373,9 @@
       <c r="CP9" s="32" t="n"/>
       <c r="CQ9" s="32" t="n"/>
       <c r="CR9" s="32" t="n"/>
-      <c r="CS9" s="32" t="n"/>
+      <c r="CS9" s="32" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CT9" s="32" t="n">
         <v>0.5</v>
       </c>
@@ -7981,7 +7983,9 @@
       <c r="CR11" s="17" t="n">
         <v>0.5</v>
       </c>
-      <c r="CS11" s="17" t="n"/>
+      <c r="CS11" s="17" t="n">
+        <v>2.25</v>
+      </c>
       <c r="CT11" s="17" t="n"/>
       <c r="CU11" s="17" t="n"/>
       <c r="CV11" s="17" t="n"/>
@@ -9733,7 +9737,9 @@
       <c r="CR17" s="32" t="n">
         <v>2.75</v>
       </c>
-      <c r="CS17" s="32" t="n"/>
+      <c r="CS17" s="32" t="n">
+        <v>2.5</v>
+      </c>
       <c r="CT17" s="32" t="n">
         <v>1.5</v>
       </c>
@@ -17536,7 +17542,9 @@
       <c r="CP45" s="17" t="n"/>
       <c r="CQ45" s="17" t="n"/>
       <c r="CR45" s="17" t="n"/>
-      <c r="CS45" s="17" t="n"/>
+      <c r="CS45" s="17" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CT45" s="17" t="n"/>
       <c r="CU45" s="17" t="n"/>
       <c r="CV45" s="17" t="n"/>
@@ -24013,7 +24021,9 @@
       <c r="CR68" s="32" t="n">
         <v>1</v>
       </c>
-      <c r="CS68" s="32" t="n"/>
+      <c r="CS68" s="32" t="n">
+        <v>1.25</v>
+      </c>
       <c r="CT68" s="32" t="n">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
Update: WMiranda_2026TimeTracking.xlsx [2026-05-21 20:20 UTC]
</commit_message>
<xml_diff>
--- a/WMiranda_2026TimeTracking.xlsx
+++ b/WMiranda_2026TimeTracking.xlsx
@@ -7381,7 +7381,9 @@
       </c>
       <c r="CU9" s="32" t="n"/>
       <c r="CV9" s="32" t="n"/>
-      <c r="CW9" s="32" t="n"/>
+      <c r="CW9" s="32" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CX9" s="32" t="n"/>
       <c r="CY9" s="32" t="n"/>
       <c r="CZ9" s="32" t="n"/>
@@ -7989,7 +7991,9 @@
       <c r="CT11" s="17" t="n"/>
       <c r="CU11" s="17" t="n"/>
       <c r="CV11" s="17" t="n"/>
-      <c r="CW11" s="17" t="n"/>
+      <c r="CW11" s="17" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CX11" s="17" t="n"/>
       <c r="CY11" s="17" t="n"/>
       <c r="CZ11" s="17" t="n"/>
@@ -9745,7 +9749,9 @@
       </c>
       <c r="CU17" s="32" t="n"/>
       <c r="CV17" s="32" t="n"/>
-      <c r="CW17" s="32" t="n"/>
+      <c r="CW17" s="32" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CX17" s="32" t="n"/>
       <c r="CY17" s="32" t="n"/>
       <c r="CZ17" s="32" t="n"/>
@@ -10871,7 +10877,9 @@
       <c r="CT21" s="17" t="n"/>
       <c r="CU21" s="17" t="n"/>
       <c r="CV21" s="17" t="n"/>
-      <c r="CW21" s="17" t="n"/>
+      <c r="CW21" s="17" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CX21" s="17" t="n"/>
       <c r="CY21" s="17" t="n"/>
       <c r="CZ21" s="17" t="n"/>
@@ -14249,7 +14257,9 @@
       </c>
       <c r="CU33" s="32" t="n"/>
       <c r="CV33" s="32" t="n"/>
-      <c r="CW33" s="32" t="n"/>
+      <c r="CW33" s="32" t="n">
+        <v>1.25</v>
+      </c>
       <c r="CX33" s="32" t="n"/>
       <c r="CY33" s="32" t="n"/>
       <c r="CZ33" s="32" t="n"/>
@@ -23655,7 +23665,9 @@
       </c>
       <c r="CU67" s="32" t="n"/>
       <c r="CV67" s="32" t="n"/>
-      <c r="CW67" s="32" t="n"/>
+      <c r="CW67" s="32" t="n">
+        <v>4</v>
+      </c>
       <c r="CX67" s="32" t="n"/>
       <c r="CY67" s="32" t="n"/>
       <c r="CZ67" s="32" t="n"/>

</xml_diff>

<commit_message>
Update: WMiranda_2026TimeTracking.xlsx [2026-05-21 20:24 UTC]
</commit_message>
<xml_diff>
--- a/WMiranda_2026TimeTracking.xlsx
+++ b/WMiranda_2026TimeTracking.xlsx
@@ -7384,7 +7384,9 @@
       <c r="CW9" s="32" t="n">
         <v>0.5</v>
       </c>
-      <c r="CX9" s="32" t="n"/>
+      <c r="CX9" s="32" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CY9" s="32" t="n"/>
       <c r="CZ9" s="32" t="n"/>
       <c r="DA9" s="32" t="n"/>
@@ -8826,7 +8828,9 @@
       <c r="CU14" s="17" t="n"/>
       <c r="CV14" s="17" t="n"/>
       <c r="CW14" s="17" t="n"/>
-      <c r="CX14" s="17" t="n"/>
+      <c r="CX14" s="17" t="n">
+        <v>1</v>
+      </c>
       <c r="CY14" s="17" t="n"/>
       <c r="CZ14" s="17" t="n"/>
       <c r="DA14" s="17" t="n"/>
@@ -9752,7 +9756,9 @@
       <c r="CW17" s="32" t="n">
         <v>1.5</v>
       </c>
-      <c r="CX17" s="32" t="n"/>
+      <c r="CX17" s="32" t="n">
+        <v>3.5</v>
+      </c>
       <c r="CY17" s="32" t="n"/>
       <c r="CZ17" s="32" t="n"/>
       <c r="DA17" s="32" t="n"/>
@@ -14260,7 +14266,9 @@
       <c r="CW33" s="32" t="n">
         <v>1.25</v>
       </c>
-      <c r="CX33" s="32" t="n"/>
+      <c r="CX33" s="32" t="n">
+        <v>2</v>
+      </c>
       <c r="CY33" s="32" t="n"/>
       <c r="CZ33" s="32" t="n"/>
       <c r="DA33" s="32" t="n"/>
@@ -26860,7 +26868,9 @@
       <c r="CU78" s="17" t="n"/>
       <c r="CV78" s="17" t="n"/>
       <c r="CW78" s="17" t="n"/>
-      <c r="CX78" s="17" t="n"/>
+      <c r="CX78" s="17" t="n">
+        <v>4</v>
+      </c>
       <c r="CY78" s="17" t="n"/>
       <c r="CZ78" s="17" t="n"/>
       <c r="DA78" s="17" t="n"/>

</xml_diff>

<commit_message>
Update: WMiranda_2026TimeTracking.xlsx [2026-05-21 20:26 UTC]
</commit_message>
<xml_diff>
--- a/WMiranda_2026TimeTracking.xlsx
+++ b/WMiranda_2026TimeTracking.xlsx
@@ -7387,7 +7387,9 @@
       <c r="CX9" s="32" t="n">
         <v>0.5</v>
       </c>
-      <c r="CY9" s="32" t="n"/>
+      <c r="CY9" s="32" t="n">
+        <v>3</v>
+      </c>
       <c r="CZ9" s="32" t="n"/>
       <c r="DA9" s="32" t="n"/>
       <c r="DB9" s="32" t="n"/>
@@ -7997,7 +7999,9 @@
         <v>1.5</v>
       </c>
       <c r="CX11" s="17" t="n"/>
-      <c r="CY11" s="17" t="n"/>
+      <c r="CY11" s="17" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CZ11" s="17" t="n"/>
       <c r="DA11" s="17" t="n"/>
       <c r="DB11" s="17" t="n"/>
@@ -9759,7 +9763,9 @@
       <c r="CX17" s="32" t="n">
         <v>3.5</v>
       </c>
-      <c r="CY17" s="32" t="n"/>
+      <c r="CY17" s="32" t="n">
+        <v>2</v>
+      </c>
       <c r="CZ17" s="32" t="n"/>
       <c r="DA17" s="32" t="n"/>
       <c r="DB17" s="32" t="n"/>
@@ -14269,7 +14275,9 @@
       <c r="CX33" s="32" t="n">
         <v>2</v>
       </c>
-      <c r="CY33" s="32" t="n"/>
+      <c r="CY33" s="32" t="n">
+        <v>2.5</v>
+      </c>
       <c r="CZ33" s="32" t="n"/>
       <c r="DA33" s="32" t="n"/>
       <c r="DB33" s="32" t="n"/>
@@ -23677,7 +23685,9 @@
         <v>4</v>
       </c>
       <c r="CX67" s="32" t="n"/>
-      <c r="CY67" s="32" t="n"/>
+      <c r="CY67" s="32" t="n">
+        <v>2.25</v>
+      </c>
       <c r="CZ67" s="32" t="n"/>
       <c r="DA67" s="32" t="n"/>
       <c r="DB67" s="32" t="n"/>

</xml_diff>